<commit_message>
sua va them profile va inter
</commit_message>
<xml_diff>
--- a/Nhom_214/TestData/Report_Nhom_214.xlsx
+++ b/Nhom_214/TestData/Report_Nhom_214.xlsx
@@ -1,31 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\C#\Nhom_214_Selenium_Test\Nhom_214\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\214_Demo\Nhom_214\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB918089-1465-4E84-94FF-2FD1A0184CFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Voucher" sheetId="7" r:id="rId1"/>
     <sheet name="Login" sheetId="8" r:id="rId2"/>
-    <sheet name="Register" sheetId="9" r:id="rId3"/>
-    <sheet name="Integration_Tests" sheetId="12" r:id="rId4"/>
-    <sheet name="RoomAdmin" sheetId="10" r:id="rId5"/>
-    <sheet name="RoomUser" sheetId="11" r:id="rId6"/>
+    <sheet name="ThongTinCN" sheetId="13" r:id="rId3"/>
+    <sheet name="Register" sheetId="9" r:id="rId4"/>
+    <sheet name="Integration_Tests" sheetId="12" r:id="rId5"/>
+    <sheet name="RoomAdmin" sheetId="10" r:id="rId6"/>
+    <sheet name="RoomUser" sheetId="11" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="196">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -216,6 +216,90 @@
     <t>Đăng nhập</t>
   </si>
   <si>
+    <t>TC_ID</t>
+  </si>
+  <si>
+    <t>NewValue</t>
+  </si>
+  <si>
+    <t>Họ tên</t>
+  </si>
+  <si>
+    <t>Số điện thoại</t>
+  </si>
+  <si>
+    <t>OldPass</t>
+  </si>
+  <si>
+    <t>NewPass</t>
+  </si>
+  <si>
+    <t>ConfirmPass</t>
+  </si>
+  <si>
+    <t>ThongTin_CN_02</t>
+  </si>
+  <si>
+    <t>edit_username</t>
+  </si>
+  <si>
+    <t>nguyenthien</t>
+  </si>
+  <si>
+    <t>Minh Thien</t>
+  </si>
+  <si>
+    <t>Cập nhật thông tin thành công!</t>
+  </si>
+  <si>
+    <t>ThongTin_CN_03</t>
+  </si>
+  <si>
+    <t>edit_email</t>
+  </si>
+  <si>
+    <t>tnc1@gmail.com</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>ThongTin_CN_08</t>
+  </si>
+  <si>
+    <t>edit_phone</t>
+  </si>
+  <si>
+    <t>Số điện thoại đã tồn tại, vui lòng nhập số khác</t>
+  </si>
+  <si>
+    <t>ThongTin_CN_10</t>
+  </si>
+  <si>
+    <t>01shsadh</t>
+  </si>
+  <si>
+    <t>Số điện thoại sai định dạng, vui lòng nhập lại</t>
+  </si>
+  <si>
+    <t>ThongTin_CN_12</t>
+  </si>
+  <si>
+    <t>change_pass</t>
+  </si>
+  <si>
+    <t>1807Tn!</t>
+  </si>
+  <si>
+    <t>Đổi mật khẩu thành công</t>
+  </si>
+  <si>
+    <t>Invalid old password</t>
+  </si>
+  <si>
+    <t>aaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaa</t>
+  </si>
+  <si>
     <t>FullName</t>
   </si>
   <si>
@@ -249,9 +333,6 @@
     <t>TREG_02</t>
   </si>
   <si>
-    <t>Minh Thien</t>
-  </si>
-  <si>
     <t>❌ Tên đăng nhập không được để trống!</t>
   </si>
   <si>
@@ -360,16 +441,16 @@
     <t>Đà Lạt</t>
   </si>
   <si>
+    <t>16/4/2026</t>
+  </si>
+  <si>
     <t>tnct@gmail.com</t>
   </si>
   <si>
     <t>Đặt phòng thành công</t>
   </si>
   <si>
-    <t>Đặt phòng thành công! Mã đặt phòng của bạn là: BK1561</t>
-  </si>
-  <si>
-    <t/>
+    <t>Đặt phòng thành công! Mã đặt phòng của bạn là: BK1570</t>
   </si>
   <si>
     <t>INT_02</t>
@@ -402,6 +483,21 @@
     <t>CHỜ XÁC NHẬN</t>
   </si>
   <si>
+    <t>INT_04</t>
+  </si>
+  <si>
+    <t>BOOKING_POPULAR</t>
+  </si>
+  <si>
+    <t>Hội An</t>
+  </si>
+  <si>
+    <t>20/05/2026</t>
+  </si>
+  <si>
+    <t>22/05/2026</t>
+  </si>
+  <si>
     <t>Param1</t>
   </si>
   <si>
@@ -501,9 +597,6 @@
     <t>Vũng Tàu</t>
   </si>
   <si>
-    <t>Link Ảnh</t>
-  </si>
-  <si>
     <t>TRU_04</t>
   </si>
   <si>
@@ -514,13 +607,19 @@
   </si>
   <si>
     <t>Load ảnh thành công</t>
+  </si>
+  <si>
+    <t>Lỗi: Thiếu thông tin đặt phòng.</t>
+  </si>
+  <si>
+    <t>17/4/2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -549,6 +648,32 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -558,7 +683,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -581,12 +706,40 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -614,11 +767,53 @@
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -922,25 +1117,25 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.33203125" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.28515625" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.44140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="40.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="40.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -978,7 +1173,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>12</v>
       </c>
@@ -1014,7 +1209,7 @@
       </c>
       <c r="L2" s="1"/>
     </row>
-    <row r="3" spans="1:12" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>19</v>
       </c>
@@ -1050,7 +1245,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>25</v>
       </c>
@@ -1076,7 +1271,7 @@
       </c>
       <c r="L4" s="5"/>
     </row>
-    <row r="5" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>29</v>
       </c>
@@ -1104,22 +1299,22 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="L3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="L3" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="9.109375" customWidth="1"/>
-    <col min="3" max="3" width="19.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="9.140625" customWidth="1"/>
+    <col min="3" max="3" width="19.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1145,7 +1340,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>39</v>
       </c>
@@ -1169,7 +1364,7 @@
       </c>
       <c r="H2" s="1"/>
     </row>
-    <row r="3" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>45</v>
       </c>
@@ -1192,14 +1387,8 @@
         <v>18</v>
       </c>
       <c r="H3" s="1"/>
-      <c r="J3" t="s">
-        <v>44</v>
-      </c>
-      <c r="K3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:8" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>48</v>
       </c>
@@ -1219,7 +1408,7 @@
       </c>
       <c r="H4" s="5"/>
     </row>
-    <row r="5" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>50</v>
       </c>
@@ -1241,7 +1430,7 @@
       </c>
       <c r="H5" s="5"/>
     </row>
-    <row r="6" spans="1:11" ht="40.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="40.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>52</v>
       </c>
@@ -1264,7 +1453,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>56</v>
       </c>
@@ -1287,7 +1476,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>60</v>
       </c>
@@ -1317,35 +1506,287 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:K9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:L7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="4" width="9.109375" customWidth="1"/>
-    <col min="5" max="5" width="13.5546875" customWidth="1"/>
+    <col min="1" max="1" width="13.140625" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" customWidth="1"/>
+    <col min="3" max="5" width="15.42578125" customWidth="1"/>
+    <col min="6" max="6" width="11.7109375" customWidth="1"/>
+    <col min="7" max="7" width="12.5703125" customWidth="1"/>
+    <col min="8" max="8" width="16.28515625" customWidth="1"/>
+    <col min="9" max="9" width="16.85546875" customWidth="1"/>
+    <col min="10" max="10" width="16.140625" customWidth="1"/>
+    <col min="11" max="11" width="9.140625" customWidth="1"/>
+    <col min="12" max="12" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="F1" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="G1" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="H1" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="K1" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="L1" s="12" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="J2" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="K2" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="L2" s="14"/>
+    </row>
+    <row r="3" spans="1:12" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="J3" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="K3" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="L3" s="14" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="62.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="E4" s="13">
+        <v>123456789</v>
+      </c>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13"/>
+      <c r="H4" s="13"/>
+      <c r="I4" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="J4" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="K4" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="L4" s="14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="F5" s="16"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="13"/>
+      <c r="I5" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="J5" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="K5" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="L5" s="14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="G6" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="H6" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="I6" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="J6" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="K6" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="L6" s="14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="86.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="G7" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="H7" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="I7" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="J7" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="K7" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="L7" s="14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="L3" r:id="rId1"/>
+    <hyperlink ref="C3" r:id="rId2"/>
+    <hyperlink ref="F6" r:id="rId3"/>
+    <hyperlink ref="F7" r:id="rId4"/>
+    <hyperlink ref="L4" r:id="rId5"/>
+    <hyperlink ref="L6" r:id="rId6"/>
+    <hyperlink ref="L7" r:id="rId7"/>
+    <hyperlink ref="L5" r:id="rId8"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="4" width="9.140625" customWidth="1"/>
+    <col min="5" max="5" width="13.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>63</v>
+        <v>91</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>33</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>64</v>
+        <v>92</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>65</v>
+        <v>93</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>34</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>66</v>
+        <v>94</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>35</v>
@@ -1360,19 +1801,19 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>67</v>
+        <v>95</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1" t="s">
-        <v>68</v>
+        <v>96</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>70</v>
+        <v>98</v>
       </c>
       <c r="F2" s="2">
         <v>12345</v>
@@ -1381,29 +1822,31 @@
         <v>12345</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>71</v>
+        <v>99</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>72</v>
+        <v>100</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="K2" s="5"/>
-    </row>
-    <row r="3" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>100</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>73</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>74</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1" t="s">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>70</v>
+        <v>98</v>
       </c>
       <c r="F3" s="2">
         <v>12345</v>
@@ -1412,31 +1855,33 @@
         <v>12345</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>71</v>
+        <v>99</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>75</v>
+        <v>102</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="K3" s="5"/>
-    </row>
-    <row r="4" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>102</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>68</v>
+        <v>96</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>78</v>
+        <v>105</v>
       </c>
       <c r="F4" s="2">
         <v>12345</v>
@@ -1445,31 +1890,33 @@
         <v>12345</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>79</v>
+        <v>106</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>80</v>
+        <v>107</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="K4" s="5"/>
-    </row>
-    <row r="5" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>107</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>81</v>
+        <v>108</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>82</v>
+        <v>109</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="F5" s="2">
         <v>12345</v>
@@ -1478,31 +1925,33 @@
         <v>12345</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>84</v>
+        <v>111</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>85</v>
+        <v>112</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="K5" s="5"/>
-    </row>
-    <row r="6" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>112</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>86</v>
+        <v>113</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>68</v>
+        <v>96</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>87</v>
+        <v>114</v>
       </c>
       <c r="F6" s="2">
         <v>12345</v>
@@ -1511,31 +1960,33 @@
         <v>12345</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>88</v>
+        <v>115</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>89</v>
+        <v>116</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="K6" s="5"/>
-    </row>
-    <row r="7" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>116</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>90</v>
+        <v>117</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>68</v>
+        <v>96</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>70</v>
+        <v>98</v>
       </c>
       <c r="F7" s="2">
         <v>12345</v>
@@ -1544,28 +1995,30 @@
         <v>54321</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>91</v>
+        <v>118</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>92</v>
+        <v>119</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="K7" s="5"/>
-    </row>
-    <row r="8" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>119</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>94</v>
+        <v>121</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>96</v>
+        <v>123</v>
       </c>
       <c r="E8" s="2">
         <v>987654321</v>
@@ -1577,31 +2030,33 @@
         <v>12345</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>97</v>
+        <v>124</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>97</v>
+        <v>124</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="K8" s="5"/>
-    </row>
-    <row r="9" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>124</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>98</v>
+        <v>125</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>99</v>
+        <v>126</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>100</v>
+        <v>127</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>100</v>
+        <v>127</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>101</v>
+        <v>128</v>
       </c>
       <c r="F9" s="2">
         <v>123456</v>
@@ -1613,47 +2068,52 @@
         <v>43</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>102</v>
+        <v>129</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="K9" s="5"/>
+        <v>129</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>18</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18D1926A-EA42-44D4-8C92-D81B9617D533}">
-  <dimension ref="A1:J4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="3" width="9.109375" customWidth="1"/>
-    <col min="4" max="5" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" customWidth="1"/>
+    <col min="3" max="3" width="12.85546875" customWidth="1"/>
+    <col min="4" max="4" width="13.42578125" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" customWidth="1"/>
+    <col min="6" max="6" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>103</v>
+        <v>130</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>104</v>
+        <v>131</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>105</v>
+        <v>132</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>106</v>
+        <v>133</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>107</v>
+        <v>134</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>35</v>
@@ -1668,357 +2128,162 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="D2" s="11">
-        <v>46026</v>
-      </c>
-      <c r="E2" s="11">
-        <v>46116</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="I2" s="1" t="s">
+    <row r="2" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>136</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>137</v>
+      </c>
+      <c r="D2" s="23" t="s">
+        <v>138</v>
+      </c>
+      <c r="E2" s="23" t="s">
+        <v>195</v>
+      </c>
+      <c r="F2" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="G2" s="18" t="s">
+        <v>140</v>
+      </c>
+      <c r="H2" s="18" t="s">
+        <v>141</v>
+      </c>
+      <c r="I2" s="18" t="s">
         <v>18</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="D3" s="11">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>143</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>144</v>
+      </c>
+      <c r="D3" s="23">
         <v>46300</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="23">
         <v>46361</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="I3" s="1" t="s">
+      <c r="F3" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="G3" s="18" t="s">
+        <v>145</v>
+      </c>
+      <c r="H3" s="18" t="s">
+        <v>145</v>
+      </c>
+      <c r="I3" s="18" t="s">
         <v>18</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="F4" s="12" t="s">
-        <v>111</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="I4" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="B4" s="19" t="s">
+        <v>147</v>
+      </c>
+      <c r="C4" s="19" t="s">
+        <v>137</v>
+      </c>
+      <c r="D4" s="24" t="s">
+        <v>148</v>
+      </c>
+      <c r="E4" s="24" t="s">
+        <v>149</v>
+      </c>
+      <c r="F4" s="20" t="s">
+        <v>139</v>
+      </c>
+      <c r="G4" s="19" t="s">
+        <v>150</v>
+      </c>
+      <c r="H4" s="19" t="s">
+        <v>151</v>
+      </c>
+      <c r="I4" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="J4" s="17" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="21" t="s">
+        <v>152</v>
+      </c>
+      <c r="B5" s="21" t="s">
+        <v>153</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>154</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>155</v>
+      </c>
+      <c r="E5" s="26" t="s">
+        <v>156</v>
+      </c>
+      <c r="F5" s="21" t="s">
+        <v>77</v>
+      </c>
+      <c r="G5" s="21" t="s">
+        <v>140</v>
+      </c>
+      <c r="H5" s="21" t="s">
+        <v>194</v>
+      </c>
+      <c r="I5" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="J4" s="5" t="s">
+      <c r="J5" s="22" t="s">
         <v>24</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="J2" r:id="rId1" xr:uid="{00000000-0004-0000-0300-000000000000}"/>
-    <hyperlink ref="J3" r:id="rId2" xr:uid="{00000000-0004-0000-0300-000001000000}"/>
-    <hyperlink ref="J4" r:id="rId3" xr:uid="{00000000-0004-0000-0300-000002000000}"/>
-    <hyperlink ref="F4" r:id="rId4" xr:uid="{00000000-0004-0000-0300-000003000000}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:L7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="2" width="9.109375" customWidth="1"/>
-    <col min="3" max="3" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="155.77734375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:12" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" ht="40.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="D2" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" ht="80.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="D3" s="2">
-        <v>1500000</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="K3" s="10"/>
-    </row>
-    <row r="4" spans="1:12" ht="80.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="D4" s="2">
-        <v>-500000</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="K4" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="L4" s="10"/>
-    </row>
-    <row r="5" spans="1:12" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="D5" s="2">
-        <v>300000</v>
-      </c>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="K5" s="5" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="C6" s="1"/>
-      <c r="D6" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="L6" s="10"/>
-    </row>
-    <row r="7" spans="1:12" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="C7" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="I7" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>114</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="K4" r:id="rId1" xr:uid="{00000000-0004-0000-0400-000000000000}"/>
-    <hyperlink ref="K5" r:id="rId2" xr:uid="{00000000-0004-0000-0400-000001000000}"/>
+    <hyperlink ref="J3" r:id="rId1"/>
+    <hyperlink ref="J4" r:id="rId2"/>
+    <hyperlink ref="F4" r:id="rId3"/>
+    <hyperlink ref="J2" r:id="rId4"/>
+    <hyperlink ref="J5" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:L7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="9.140625" customWidth="1"/>
+    <col min="3" max="3" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="155.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2026,109 +2291,334 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>104</v>
+        <v>157</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" ht="40.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>30</v>
+        <v>163</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>18</v>
-      </c>
+        <v>164</v>
+      </c>
+      <c r="D2" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
       <c r="G2" s="1"/>
-    </row>
-    <row r="3" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H2" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="80.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>30</v>
+        <v>166</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>154</v>
+        <v>167</v>
+      </c>
+      <c r="D3" s="2">
+        <v>1500000</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>155</v>
+        <v>168</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="G3" s="1"/>
-    </row>
-    <row r="4" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>169</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K3" s="10" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="80.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>156</v>
+        <v>172</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>30</v>
+        <v>166</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>154</v>
+        <v>167</v>
+      </c>
+      <c r="D4" s="2">
+        <v>-500000</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>155</v>
+        <v>168</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>169</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L4" s="10"/>
+    </row>
+    <row r="5" spans="1:12" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>159</v>
+        <v>174</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>18</v>
-      </c>
+        <v>175</v>
+      </c>
+      <c r="D5" s="2">
+        <v>300000</v>
+      </c>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
       <c r="G5" s="1"/>
+      <c r="H5" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="C6" s="1"/>
+      <c r="D6" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="L6" s="10"/>
+    </row>
+    <row r="7" spans="1:12" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="C7" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>78</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="G4" r:id="rId1" xr:uid="{00000000-0004-0000-0500-000000000000}"/>
+    <hyperlink ref="K4" r:id="rId1"/>
+    <hyperlink ref="K5" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" s="1"/>
+    </row>
+    <row r="3" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="1"/>
+    </row>
+    <row r="4" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>